<commit_message>
feat: 2026년 신규 논문 2건(PUB-135, PUB-136) 추가 및 논문 통계(128건) 동기화
</commit_message>
<xml_diff>
--- a/data/publications.xlsx
+++ b/data/publications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SmartCity20\.gemini\antigravity\scratch\surd-lab-homepage\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686A9505-5DA0-494C-BC72-76650D6F07B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB47416-67D1-4DB5-ACE8-F5ACAF9990ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25800" yWindow="0" windowWidth="25800" windowHeight="21000" xr2:uid="{FB3B5A28-B30A-4FB9-B973-DA7691D44842}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25800" windowHeight="21000" xr2:uid="{FB3B5A28-B30A-4FB9-B973-DA7691D44842}"/>
   </bookViews>
   <sheets>
     <sheet name="publications" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1410" uniqueCount="604">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1430" uniqueCount="614">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2186,6 +2186,43 @@
   <si>
     <t>type_index</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PUB-135</t>
+  </si>
+  <si>
+    <t>류준영, 남진</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>산업단지 재생을 위한 공공투자 거버넌스 효율화 방안 연구: 한국과 일본의 운용 모델 비교를 중심으로</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>223-346</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026, 류준영, 남진, 산업단지 재생을 위한 공공투자 거버넌스 효율화 방안 연구 _ 한국과 일본의 운용 모델 비교를 중심으로, 도시부동산연구, 17(1), 223-246</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PUB-136</t>
+  </si>
+  <si>
+    <t>이채은, 남진</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울시 청년안심주택 입지 유형화 및 특성 분석에 관한 연구</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>95-119</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026, 이채은, 남진, 서울시 청년안심주택 입지 유형화 및 특성 분석에 관한 연구, 도시부동산연구, 17(2), 95-119</t>
   </si>
 </sst>
 </file>
@@ -2241,7 +2278,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2252,6 +2289,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2292,8 +2332,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3B219D66-BA1A-4F2C-94F2-DC6495E11B62}" name="PublicationsTable" displayName="PublicationsTable" ref="A1:Q135" totalsRowShown="0">
-  <autoFilter ref="A1:Q135" xr:uid="{3B219D66-BA1A-4F2C-94F2-DC6495E11B62}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3B219D66-BA1A-4F2C-94F2-DC6495E11B62}" name="PublicationsTable" displayName="PublicationsTable" ref="A1:Q137" totalsRowShown="0">
+  <autoFilter ref="A1:Q137" xr:uid="{3B219D66-BA1A-4F2C-94F2-DC6495E11B62}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{A3F79930-0951-4BB1-9334-E9583C167FB9}" name="id"/>
     <tableColumn id="2" xr3:uid="{E3831AFD-57F7-42F7-9B92-611D56962AE7}" name="type"/>
@@ -2646,7 +2686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDD90BD3-3697-404D-A251-253A8639131A}">
-  <dimension ref="A1:Q135"/>
+  <dimension ref="A1:Q137"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="12.125" customWidth="1"/>
@@ -8014,16 +8054,100 @@
         <v>287</v>
       </c>
     </row>
+    <row r="136" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>604</v>
+      </c>
+      <c r="B136" t="s">
+        <v>285</v>
+      </c>
+      <c r="C136" t="s">
+        <v>600</v>
+      </c>
+      <c r="D136">
+        <f>VALUE(LEFT(PublicationsTable[[#This Row],[file_name]],4))</f>
+        <v>2026</v>
+      </c>
+      <c r="E136" t="s">
+        <v>605</v>
+      </c>
+      <c r="F136" t="s">
+        <v>606</v>
+      </c>
+      <c r="G136" t="s">
+        <v>533</v>
+      </c>
+      <c r="H136">
+        <v>17</v>
+      </c>
+      <c r="I136">
+        <v>1</v>
+      </c>
+      <c r="J136" t="s">
+        <v>607</v>
+      </c>
+      <c r="M136" t="s">
+        <v>434</v>
+      </c>
+      <c r="O136" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="P136" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="137" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>609</v>
+      </c>
+      <c r="B137" t="s">
+        <v>285</v>
+      </c>
+      <c r="C137" t="s">
+        <v>600</v>
+      </c>
+      <c r="D137">
+        <f>VALUE(LEFT(PublicationsTable[[#This Row],[file_name]],4))</f>
+        <v>2026</v>
+      </c>
+      <c r="E137" t="s">
+        <v>610</v>
+      </c>
+      <c r="F137" t="s">
+        <v>611</v>
+      </c>
+      <c r="G137" t="s">
+        <v>533</v>
+      </c>
+      <c r="H137">
+        <v>17</v>
+      </c>
+      <c r="I137">
+        <v>2</v>
+      </c>
+      <c r="J137" t="s">
+        <v>612</v>
+      </c>
+      <c r="M137" t="s">
+        <v>434</v>
+      </c>
+      <c r="O137" s="4" t="s">
+        <v>613</v>
+      </c>
+      <c r="P137" t="s">
+        <v>287</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B135" xr:uid="{4097AEAF-A1C2-4390-9B06-0AF57FD443A1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B137" xr:uid="{4097AEAF-A1C2-4390-9B06-0AF57FD443A1}">
       <formula1>"Journal,Conference,Book,Report"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C135" xr:uid="{DF9A1197-E5D4-4C18-8B8C-E3B493C707CA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C137" xr:uid="{DF9A1197-E5D4-4C18-8B8C-E3B493C707CA}">
       <formula1>"SSCI,SCIE,KCI,Other,Unverified,Not applicable"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P135 M2:M135" xr:uid="{24D29147-F31F-48DB-8F1C-55C5A592175F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P137 M2:M137" xr:uid="{24D29147-F31F-48DB-8F1C-55C5A592175F}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>